<commit_message>
Renamed pull button to Recovery for better clarity.
Renamed Purge Logs to Purge Shared Logs for better clarity
</commit_message>
<xml_diff>
--- a/output/chapter4/Survey-Response-Entry-Template.xlsx
+++ b/output/chapter4/Survey-Response-Entry-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justine mendoza\source\repos\NFC_System\output\chapter4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3174941B-E23E-459E-BCA5-1EC3371C5685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8340CE13-FF1C-40A7-8D36-CBB8B749CDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -976,10 +976,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1202,28 +1202,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.95" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="16" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1919,11 +1919,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A33:H33"/>
@@ -1933,6 +1928,11 @@
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9694,34 +9694,34 @@
       <c r="A77" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B77" s="16" t="s">
+      <c r="B77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="C77" s="16" t="s">
+      <c r="C77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D77" s="16" t="s">
+      <c r="D77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="E77" s="16" t="s">
+      <c r="E77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="F77" s="16" t="s">
+      <c r="F77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="G77" s="16" t="s">
+      <c r="G77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="H77" s="16" t="s">
+      <c r="H77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="I77" s="16" t="s">
+      <c r="I77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="J77" s="16" t="s">
+      <c r="J77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="K77" s="16" t="s">
+      <c r="K77" s="15" t="s">
         <v>132</v>
       </c>
       <c r="L77" s="1"/>
@@ -11279,26 +11279,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A74:K74"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="B77:K77"/>
-    <mergeCell ref="B78:K78"/>
-    <mergeCell ref="B79:K79"/>
-    <mergeCell ref="B80:K80"/>
-    <mergeCell ref="B81:K81"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="B83:K83"/>
-    <mergeCell ref="B84:K84"/>
-    <mergeCell ref="B85:K85"/>
-    <mergeCell ref="B86:K86"/>
-    <mergeCell ref="B87:K87"/>
-    <mergeCell ref="B88:K88"/>
-    <mergeCell ref="B89:K89"/>
-    <mergeCell ref="B90:K90"/>
-    <mergeCell ref="B91:K91"/>
-    <mergeCell ref="B92:K92"/>
-    <mergeCell ref="B93:K93"/>
-    <mergeCell ref="B94:K94"/>
     <mergeCell ref="B100:K100"/>
     <mergeCell ref="B101:K101"/>
     <mergeCell ref="A103:K103"/>
@@ -11307,6 +11287,26 @@
     <mergeCell ref="B97:K97"/>
     <mergeCell ref="B98:K98"/>
     <mergeCell ref="B99:K99"/>
+    <mergeCell ref="B90:K90"/>
+    <mergeCell ref="B91:K91"/>
+    <mergeCell ref="B92:K92"/>
+    <mergeCell ref="B93:K93"/>
+    <mergeCell ref="B94:K94"/>
+    <mergeCell ref="B85:K85"/>
+    <mergeCell ref="B86:K86"/>
+    <mergeCell ref="B87:K87"/>
+    <mergeCell ref="B88:K88"/>
+    <mergeCell ref="B89:K89"/>
+    <mergeCell ref="B80:K80"/>
+    <mergeCell ref="B81:K81"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="B83:K83"/>
+    <mergeCell ref="B84:K84"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="B77:K77"/>
+    <mergeCell ref="B78:K78"/>
+    <mergeCell ref="B79:K79"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -19069,34 +19069,34 @@
       <c r="A77" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B77" s="16" t="s">
+      <c r="B77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="C77" s="16" t="s">
+      <c r="C77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D77" s="16" t="s">
+      <c r="D77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="E77" s="16" t="s">
+      <c r="E77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="F77" s="16" t="s">
+      <c r="F77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="G77" s="16" t="s">
+      <c r="G77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="H77" s="16" t="s">
+      <c r="H77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="I77" s="16" t="s">
+      <c r="I77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="J77" s="16" t="s">
+      <c r="J77" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="K77" s="16" t="s">
+      <c r="K77" s="15" t="s">
         <v>132</v>
       </c>
       <c r="L77" s="1"/>
@@ -20654,26 +20654,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A74:K74"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="B77:K77"/>
-    <mergeCell ref="B78:K78"/>
-    <mergeCell ref="B79:K79"/>
-    <mergeCell ref="B80:K80"/>
-    <mergeCell ref="B81:K81"/>
-    <mergeCell ref="B82:K82"/>
-    <mergeCell ref="B83:K83"/>
-    <mergeCell ref="B84:K84"/>
-    <mergeCell ref="B85:K85"/>
-    <mergeCell ref="B86:K86"/>
-    <mergeCell ref="B87:K87"/>
-    <mergeCell ref="B88:K88"/>
-    <mergeCell ref="B89:K89"/>
-    <mergeCell ref="B90:K90"/>
-    <mergeCell ref="B91:K91"/>
-    <mergeCell ref="B92:K92"/>
-    <mergeCell ref="B93:K93"/>
-    <mergeCell ref="B94:K94"/>
     <mergeCell ref="B100:K100"/>
     <mergeCell ref="B101:K101"/>
     <mergeCell ref="A103:K103"/>
@@ -20682,6 +20662,26 @@
     <mergeCell ref="B97:K97"/>
     <mergeCell ref="B98:K98"/>
     <mergeCell ref="B99:K99"/>
+    <mergeCell ref="B90:K90"/>
+    <mergeCell ref="B91:K91"/>
+    <mergeCell ref="B92:K92"/>
+    <mergeCell ref="B93:K93"/>
+    <mergeCell ref="B94:K94"/>
+    <mergeCell ref="B85:K85"/>
+    <mergeCell ref="B86:K86"/>
+    <mergeCell ref="B87:K87"/>
+    <mergeCell ref="B88:K88"/>
+    <mergeCell ref="B89:K89"/>
+    <mergeCell ref="B80:K80"/>
+    <mergeCell ref="B81:K81"/>
+    <mergeCell ref="B82:K82"/>
+    <mergeCell ref="B83:K83"/>
+    <mergeCell ref="B84:K84"/>
+    <mergeCell ref="A74:K74"/>
+    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="B77:K77"/>
+    <mergeCell ref="B78:K78"/>
+    <mergeCell ref="B79:K79"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>